<commit_message>
Actualización diaria automática de ETFs Morningstar
</commit_message>
<xml_diff>
--- a/lista_completa_etfs_morningstar.xlsx
+++ b/lista_completa_etfs_morningstar.xlsx
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>745.76</v>
+        <v>744.78</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -571,7 +571,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>725.17</v>
+        <v>712.6044000000001</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -630,7 +630,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>299.32</v>
+        <v>297.58</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>66.48</v>
+        <v>65.7</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -748,7 +748,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>87.77</v>
+        <v>89.34999999999999</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -807,7 +807,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>96.08</v>
+        <v>97.3</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -866,7 +866,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>369.27</v>
+        <v>368.76</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -925,7 +925,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>685.46</v>
+        <v>684.84</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -984,7 +984,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>156.12</v>
+        <v>156.15</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -1043,7 +1043,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>125.23</v>
+        <v>125.74</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1171,7 +1171,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>211</v>
+        <v>212.7</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -1230,7 +1230,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>318.6</v>
+        <v>320.7</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -1293,7 +1293,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>295.25</v>
+        <v>297</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -1415,7 +1415,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>13.845</v>
+        <v>13.965</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -1474,7 +1474,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>20.64</v>
+        <v>20.735</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -1533,7 +1533,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>5576</v>
+        <v>5595.25</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -1661,7 +1661,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>47.383</v>
+        <v>48.38</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -1726,7 +1726,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>89.928</v>
+        <v>90.316</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -1854,7 +1854,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>22.44</v>
+        <v>22.74</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1917,7 +1917,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>3.549</v>
+        <v>3.55</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>

</xml_diff>